<commit_message>
taper historical data, fix RL underdog logic
</commit_message>
<xml_diff>
--- a/reports/picks_tracker.xlsx
+++ b/reports/picks_tracker.xlsx
@@ -801,17 +801,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>ATL</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>55.8%</t>
+          <t>50.3%</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>5.6-5.9</t>
+          <t>5.2-5.5</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.31</v>
+        <v>0.24</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="L2" s="2" t="n">
-        <v>11.5</v>
+        <v>10.7</v>
       </c>
       <c r="M2" s="4" t="n">
         <v>8.5</v>
@@ -882,12 +882,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>57.2%</t>
+          <t>58.6%</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>4.0-4.1</t>
+          <t>4.4-4.3</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="J3" s="6" t="n">
-        <v>0.16</v>
+        <v>-0.06</v>
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="L3" s="6" t="n">
-        <v>8.1</v>
+        <v>8.6</v>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
@@ -960,12 +960,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>66.8%</t>
+          <t>65.0%</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>3.8-5.7</t>
+          <t>3.8-5.4</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -979,15 +979,15 @@
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1.95</v>
+        <v>1.55</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>9.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>7.5</v>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>48.1%</t>
+          <t>46.5%</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>4.3-4.9</t>
+          <t>4.0-5.1</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -1055,15 +1055,15 @@
         </is>
       </c>
       <c r="J5" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>1.17</v>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="L5" s="6" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
@@ -1109,17 +1109,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>57.5%</t>
+          <t>54.1%</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>5.7-4.7</t>
+          <t>5.8-4.4</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>-0.99</v>
+        <v>-1.43</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>10.4</v>
+        <v>10.2</v>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
@@ -1187,17 +1187,17 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>35.5%</t>
+          <t>45.8%</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>6.3-5.1</t>
+          <t>5.5-5.0</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
@@ -1207,11 +1207,11 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>NYM +1.5</t>
         </is>
       </c>
       <c r="J7" s="6" t="n">
-        <v>-1.22</v>
+        <v>-0.48</v>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
         </is>
       </c>
       <c r="L7" s="6" t="n">
-        <v>11.4</v>
+        <v>10.5</v>
       </c>
       <c r="M7" s="4" t="n">
         <v>7.5</v>
@@ -1263,17 +1263,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>MIA</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>53.4%</t>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>47.4%</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>4.9-5.2</t>
+          <t>5.1-4.7</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1283,11 +1283,11 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>STL +1.5</t>
+          <t>MIA +1.5</t>
         </is>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0.21</v>
+        <v>-0.42</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="L8" s="2" t="n">
-        <v>10.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="M8" s="4" t="n">
         <v>8.5</v>
@@ -1339,17 +1339,17 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>TOR</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>46.1%</t>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>51.1%</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>3.8-5.3</t>
+          <t>3.8-5.2</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>LAA +1.5</t>
+          <t>TOR +1.5</t>
         </is>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1.53</v>
+        <v>1.46</v>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="L9" s="6" t="n">
-        <v>9.1</v>
+        <v>9</v>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
@@ -1422,12 +1422,12 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>41.9%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>4.8-4.0</t>
+          <t>4.7-4.3</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="J10" s="2" t="n">
-        <v>-0.84</v>
+        <v>-0.49</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1449,7 +1449,7 @@
         </is>
       </c>
       <c r="L10" s="2" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="M10" s="4" t="n">
         <v>9</v>
@@ -1493,17 +1493,17 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>54.7%</t>
+          <t>53.9%</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>3.7-5.2</t>
+          <t>4.0-5.1</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="J11" s="6" t="n">
-        <v>1.48</v>
+        <v>1.11</v>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="L11" s="6" t="n">
-        <v>8.9</v>
+        <v>9.1</v>
       </c>
       <c r="M11" s="4" t="n">
         <v>8.5</v>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>65.5%</t>
+          <t>63.2%</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>4.0-4.6</t>
+          <t>4.1-4.7</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1601,7 +1601,7 @@
         </is>
       </c>
       <c r="L12" s="2" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
@@ -1652,12 +1652,12 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>74.0%</t>
+          <t>74.5%</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>3.7-5.5</t>
+          <t>3.7-5.4</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="J13" s="6" t="n">
-        <v>1.83</v>
+        <v>1.71</v>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="L13" s="6" t="n">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="M13" s="4" t="n">
         <v>8</v>
@@ -1728,12 +1728,12 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>79.8%</t>
+          <t>76.2%</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>3.2-5.4</t>
+          <t>3.7-5.6</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="J14" s="2" t="n">
-        <v>2.14</v>
+        <v>1.94</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
@@ -1755,10 +1755,10 @@
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>8.6</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
@@ -1802,14 +1802,14 @@
           <t>BOS</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>60.2%</t>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>54.0%</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>3.9-5.7</t>
+          <t>3.9-5.1</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -1819,19 +1819,19 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>BOS -1.5</t>
+          <t>NYY +1.5</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>1.72</v>
+        <v>1.25</v>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>OVER</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L15" s="6" t="n">
-        <v>9.6</v>
+        <v>9</v>
       </c>
       <c r="M15" s="4" t="n">
         <v>8.5</v>
@@ -1880,12 +1880,12 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>48.9%</t>
+          <t>48.6%</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>4.3-4.7</t>
+          <t>4.3-4.6</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1899,11 +1899,11 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.44</v>
+        <v>0.3</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>OVER</t>
         </is>
       </c>
       <c r="L16" s="2" t="n">

</xml_diff>